<commit_message>
parent access to own child data
</commit_message>
<xml_diff>
--- a/dc-uat-checklist.xlsx
+++ b/dc-uat-checklist.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\daycare-system\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49964668-5574-4B06-9A52-3BCB33A87CD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8196" tabRatio="500" activeTab="2"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -18,8 +24,17 @@
     <definedName name="_xlnm.Print_Area" localSheetId="2">'UAT Checklist'!$A$1:$K$111</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'UAT Checklist'!$1:$1</definedName>
   </definedNames>
-  <calcPr calcId="144525" iterateDelta="1E-4"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -1584,7 +1599,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1701,13 +1716,6 @@
   <dxfs count="5">
     <dxf>
       <font>
-        <b/>
-        <color rgb="FFA32D2D"/>
-        <name val="Arial"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF5F5E5A"/>
         <name val="Arial"/>
       </font>
@@ -1752,6 +1760,13 @@
           <bgColor rgb="FFD9F2E6"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFA32D2D"/>
+        <name val="Arial"/>
+      </font>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1826,6 +1841,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -2009,127 +2027,127 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:B26"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" ht="21" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:2" ht="20" x14ac:dyDescent="0.4">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B5" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B6" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B7" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B8" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B9" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B10" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B11" s="4"/>
     </row>
-    <row r="12" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B12" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B13" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B14" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B15" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B16" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B17" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B18" s="4"/>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B19" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B20" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B21" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B22" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B23" s="4"/>
     </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B24" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B25" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B26" s="4" t="s">
         <v>20</v>
       </c>
@@ -2141,12 +2159,12 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:I27"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
@@ -2154,17 +2172,17 @@
     <col min="9" max="9" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" ht="21" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:9" ht="20" x14ac:dyDescent="0.4">
       <c r="B2" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B3" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B5" s="5" t="s">
         <v>23</v>
       </c>
@@ -2190,7 +2208,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B6" s="6" t="s">
         <v>31</v>
       </c>
@@ -2223,7 +2241,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B7" s="6" t="s">
         <v>32</v>
       </c>
@@ -2256,7 +2274,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B8" s="6" t="s">
         <v>33</v>
       </c>
@@ -2266,11 +2284,11 @@
       </c>
       <c r="D8" s="6">
         <f>COUNTIFS('UAT Checklist'!$B$2:$B$111,$B8,'UAT Checklist'!$H$2:$H$111,"Not Tested")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E8" s="6">
         <f>COUNTIFS('UAT Checklist'!$B$2:$B$111,$B8,'UAT Checklist'!$H$2:$H$111,"Pass")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="6">
         <f>COUNTIFS('UAT Checklist'!$B$2:$B$111,$B8,'UAT Checklist'!$H$2:$H$111,"Fail")</f>
@@ -2286,10 +2304,10 @@
       </c>
       <c r="I8" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.3">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B9" s="6" t="s">
         <v>34</v>
       </c>
@@ -2322,7 +2340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B10" s="6" t="s">
         <v>35</v>
       </c>
@@ -2355,7 +2373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B11" s="6" t="s">
         <v>36</v>
       </c>
@@ -2388,7 +2406,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B12" s="6" t="s">
         <v>37</v>
       </c>
@@ -2421,7 +2439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B13" s="6" t="s">
         <v>38</v>
       </c>
@@ -2454,7 +2472,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B14" s="6" t="s">
         <v>39</v>
       </c>
@@ -2487,7 +2505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B15" s="6" t="s">
         <v>40</v>
       </c>
@@ -2520,7 +2538,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B16" s="6" t="s">
         <v>41</v>
       </c>
@@ -2553,7 +2571,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B17" s="6" t="s">
         <v>42</v>
       </c>
@@ -2586,7 +2604,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B18" s="6" t="s">
         <v>43</v>
       </c>
@@ -2619,7 +2637,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B19" s="6" t="s">
         <v>44</v>
       </c>
@@ -2652,7 +2670,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B20" s="6" t="s">
         <v>45</v>
       </c>
@@ -2685,7 +2703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B21" s="6" t="s">
         <v>46</v>
       </c>
@@ -2718,7 +2736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B22" s="6" t="s">
         <v>47</v>
       </c>
@@ -2751,7 +2769,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B23" s="6" t="s">
         <v>48</v>
       </c>
@@ -2784,7 +2802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B24" s="6" t="s">
         <v>49</v>
       </c>
@@ -2817,7 +2835,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B25" s="6" t="s">
         <v>50</v>
       </c>
@@ -2850,7 +2868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B26" s="6" t="s">
         <v>51</v>
       </c>
@@ -2883,7 +2901,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B27" s="8" t="s">
         <v>52</v>
       </c>
@@ -2893,11 +2911,11 @@
       </c>
       <c r="D27" s="8">
         <f t="shared" si="1"/>
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E27" s="8">
         <f t="shared" si="1"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F27" s="8">
         <f t="shared" si="1"/>
@@ -2913,7 +2931,7 @@
       </c>
       <c r="I27" s="9">
         <f t="shared" si="0"/>
-        <v>0.10909090909090909</v>
+        <v>0.11818181818181818</v>
       </c>
     </row>
   </sheetData>
@@ -2935,15 +2953,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:K111"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="15.6640625" customWidth="1"/>
+    <col min="2" max="2" width="15.6328125" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
     <col min="5" max="5" width="45" customWidth="1"/>
@@ -2955,7 +2973,7 @@
     <col min="11" max="11" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>53</v>
       </c>
@@ -2990,7 +3008,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="59.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="59.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="10">
         <v>1</v>
       </c>
@@ -3021,7 +3039,7 @@
       <c r="J2" s="10"/>
       <c r="K2" s="10"/>
     </row>
-    <row r="3" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="10">
         <v>2</v>
       </c>
@@ -3050,7 +3068,7 @@
       <c r="J3" s="10"/>
       <c r="K3" s="10"/>
     </row>
-    <row r="4" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="10">
         <v>3</v>
       </c>
@@ -3079,7 +3097,7 @@
       <c r="J4" s="10"/>
       <c r="K4" s="10"/>
     </row>
-    <row r="5" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="10">
         <v>4</v>
       </c>
@@ -3108,7 +3126,7 @@
       <c r="J5" s="10"/>
       <c r="K5" s="10"/>
     </row>
-    <row r="6" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="10">
         <v>5</v>
       </c>
@@ -3137,7 +3155,7 @@
       <c r="J6" s="10"/>
       <c r="K6" s="10"/>
     </row>
-    <row r="7" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="10">
         <v>6</v>
       </c>
@@ -3166,7 +3184,7 @@
       <c r="J7" s="10"/>
       <c r="K7" s="10"/>
     </row>
-    <row r="8" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="10">
         <v>7</v>
       </c>
@@ -3195,7 +3213,7 @@
       <c r="J8" s="10"/>
       <c r="K8" s="10"/>
     </row>
-    <row r="9" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="10">
         <v>8</v>
       </c>
@@ -3224,7 +3242,7 @@
       <c r="J9" s="10"/>
       <c r="K9" s="10"/>
     </row>
-    <row r="10" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="10">
         <v>9</v>
       </c>
@@ -3253,7 +3271,7 @@
       <c r="J10" s="10"/>
       <c r="K10" s="10"/>
     </row>
-    <row r="11" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="10">
         <v>10</v>
       </c>
@@ -3282,7 +3300,7 @@
       <c r="J11" s="10"/>
       <c r="K11" s="10"/>
     </row>
-    <row r="12" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="10">
         <v>11</v>
       </c>
@@ -3311,7 +3329,7 @@
       <c r="J12" s="10"/>
       <c r="K12" s="10"/>
     </row>
-    <row r="13" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="10">
         <v>12</v>
       </c>
@@ -3340,7 +3358,7 @@
       <c r="J13" s="10"/>
       <c r="K13" s="10"/>
     </row>
-    <row r="14" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="10">
         <v>13</v>
       </c>
@@ -3369,7 +3387,7 @@
       <c r="J14" s="10"/>
       <c r="K14" s="10"/>
     </row>
-    <row r="15" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="10">
         <v>14</v>
       </c>
@@ -3398,7 +3416,7 @@
       <c r="J15" s="10"/>
       <c r="K15" s="10"/>
     </row>
-    <row r="16" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="10">
         <v>15</v>
       </c>
@@ -3421,13 +3439,13 @@
         <v>76</v>
       </c>
       <c r="H16" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I16" s="11"/>
       <c r="J16" s="10"/>
       <c r="K16" s="10"/>
     </row>
-    <row r="17" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="10">
         <v>16</v>
       </c>
@@ -3456,7 +3474,7 @@
       <c r="J17" s="10"/>
       <c r="K17" s="10"/>
     </row>
-    <row r="18" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="10">
         <v>17</v>
       </c>
@@ -3485,7 +3503,7 @@
       <c r="J18" s="10"/>
       <c r="K18" s="10"/>
     </row>
-    <row r="19" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="10">
         <v>18</v>
       </c>
@@ -3514,7 +3532,7 @@
       <c r="J19" s="10"/>
       <c r="K19" s="10"/>
     </row>
-    <row r="20" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="10">
         <v>19</v>
       </c>
@@ -3543,7 +3561,7 @@
       <c r="J20" s="10"/>
       <c r="K20" s="10"/>
     </row>
-    <row r="21" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="10">
         <v>20</v>
       </c>
@@ -3572,7 +3590,7 @@
       <c r="J21" s="10"/>
       <c r="K21" s="10"/>
     </row>
-    <row r="22" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="10">
         <v>21</v>
       </c>
@@ -3601,7 +3619,7 @@
       <c r="J22" s="10"/>
       <c r="K22" s="10"/>
     </row>
-    <row r="23" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="10">
         <v>22</v>
       </c>
@@ -3630,7 +3648,7 @@
       <c r="J23" s="10"/>
       <c r="K23" s="10"/>
     </row>
-    <row r="24" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="10">
         <v>23</v>
       </c>
@@ -3659,7 +3677,7 @@
       <c r="J24" s="10"/>
       <c r="K24" s="10"/>
     </row>
-    <row r="25" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="10">
         <v>24</v>
       </c>
@@ -3688,7 +3706,7 @@
       <c r="J25" s="10"/>
       <c r="K25" s="10"/>
     </row>
-    <row r="26" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="10">
         <v>25</v>
       </c>
@@ -3717,7 +3735,7 @@
       <c r="J26" s="10"/>
       <c r="K26" s="10"/>
     </row>
-    <row r="27" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="10">
         <v>26</v>
       </c>
@@ -3746,7 +3764,7 @@
       <c r="J27" s="10"/>
       <c r="K27" s="10"/>
     </row>
-    <row r="28" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="10">
         <v>27</v>
       </c>
@@ -3775,7 +3793,7 @@
       <c r="J28" s="10"/>
       <c r="K28" s="10"/>
     </row>
-    <row r="29" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="10">
         <v>28</v>
       </c>
@@ -3804,7 +3822,7 @@
       <c r="J29" s="10"/>
       <c r="K29" s="10"/>
     </row>
-    <row r="30" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="10">
         <v>29</v>
       </c>
@@ -3833,7 +3851,7 @@
       <c r="J30" s="10"/>
       <c r="K30" s="10"/>
     </row>
-    <row r="31" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="10">
         <v>30</v>
       </c>
@@ -3862,7 +3880,7 @@
       <c r="J31" s="10"/>
       <c r="K31" s="10"/>
     </row>
-    <row r="32" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="10">
         <v>31</v>
       </c>
@@ -3891,7 +3909,7 @@
       <c r="J32" s="10"/>
       <c r="K32" s="10"/>
     </row>
-    <row r="33" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="10">
         <v>32</v>
       </c>
@@ -3920,7 +3938,7 @@
       <c r="J33" s="10"/>
       <c r="K33" s="10"/>
     </row>
-    <row r="34" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="10">
         <v>33</v>
       </c>
@@ -3949,7 +3967,7 @@
       <c r="J34" s="10"/>
       <c r="K34" s="10"/>
     </row>
-    <row r="35" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="10">
         <v>34</v>
       </c>
@@ -3978,7 +3996,7 @@
       <c r="J35" s="10"/>
       <c r="K35" s="10"/>
     </row>
-    <row r="36" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="10">
         <v>35</v>
       </c>
@@ -4007,7 +4025,7 @@
       <c r="J36" s="10"/>
       <c r="K36" s="10"/>
     </row>
-    <row r="37" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="10">
         <v>36</v>
       </c>
@@ -4036,7 +4054,7 @@
       <c r="J37" s="10"/>
       <c r="K37" s="10"/>
     </row>
-    <row r="38" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="10">
         <v>37</v>
       </c>
@@ -4065,7 +4083,7 @@
       <c r="J38" s="10"/>
       <c r="K38" s="10"/>
     </row>
-    <row r="39" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="10">
         <v>38</v>
       </c>
@@ -4094,7 +4112,7 @@
       <c r="J39" s="10"/>
       <c r="K39" s="10"/>
     </row>
-    <row r="40" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="10">
         <v>39</v>
       </c>
@@ -4123,7 +4141,7 @@
       <c r="J40" s="10"/>
       <c r="K40" s="10"/>
     </row>
-    <row r="41" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="10">
         <v>40</v>
       </c>
@@ -4152,7 +4170,7 @@
       <c r="J41" s="10"/>
       <c r="K41" s="10"/>
     </row>
-    <row r="42" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="10">
         <v>41</v>
       </c>
@@ -4181,7 +4199,7 @@
       <c r="J42" s="10"/>
       <c r="K42" s="10"/>
     </row>
-    <row r="43" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="10">
         <v>42</v>
       </c>
@@ -4210,7 +4228,7 @@
       <c r="J43" s="10"/>
       <c r="K43" s="10"/>
     </row>
-    <row r="44" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="10">
         <v>43</v>
       </c>
@@ -4239,7 +4257,7 @@
       <c r="J44" s="10"/>
       <c r="K44" s="10"/>
     </row>
-    <row r="45" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="10">
         <v>44</v>
       </c>
@@ -4268,7 +4286,7 @@
       <c r="J45" s="10"/>
       <c r="K45" s="10"/>
     </row>
-    <row r="46" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="10">
         <v>45</v>
       </c>
@@ -4297,7 +4315,7 @@
       <c r="J46" s="10"/>
       <c r="K46" s="10"/>
     </row>
-    <row r="47" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="10">
         <v>46</v>
       </c>
@@ -4326,7 +4344,7 @@
       <c r="J47" s="10"/>
       <c r="K47" s="10"/>
     </row>
-    <row r="48" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="10">
         <v>47</v>
       </c>
@@ -4355,7 +4373,7 @@
       <c r="J48" s="10"/>
       <c r="K48" s="10"/>
     </row>
-    <row r="49" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="10">
         <v>48</v>
       </c>
@@ -4384,7 +4402,7 @@
       <c r="J49" s="10"/>
       <c r="K49" s="10"/>
     </row>
-    <row r="50" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="10">
         <v>49</v>
       </c>
@@ -4413,7 +4431,7 @@
       <c r="J50" s="10"/>
       <c r="K50" s="10"/>
     </row>
-    <row r="51" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="10">
         <v>50</v>
       </c>
@@ -4442,7 +4460,7 @@
       <c r="J51" s="10"/>
       <c r="K51" s="10"/>
     </row>
-    <row r="52" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="10">
         <v>51</v>
       </c>
@@ -4471,7 +4489,7 @@
       <c r="J52" s="10"/>
       <c r="K52" s="10"/>
     </row>
-    <row r="53" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="10">
         <v>52</v>
       </c>
@@ -4500,7 +4518,7 @@
       <c r="J53" s="10"/>
       <c r="K53" s="10"/>
     </row>
-    <row r="54" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="10">
         <v>53</v>
       </c>
@@ -4529,7 +4547,7 @@
       <c r="J54" s="10"/>
       <c r="K54" s="10"/>
     </row>
-    <row r="55" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="10">
         <v>54</v>
       </c>
@@ -4558,7 +4576,7 @@
       <c r="J55" s="10"/>
       <c r="K55" s="10"/>
     </row>
-    <row r="56" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="10">
         <v>55</v>
       </c>
@@ -4587,7 +4605,7 @@
       <c r="J56" s="10"/>
       <c r="K56" s="10"/>
     </row>
-    <row r="57" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="10">
         <v>56</v>
       </c>
@@ -4616,7 +4634,7 @@
       <c r="J57" s="10"/>
       <c r="K57" s="10"/>
     </row>
-    <row r="58" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="10">
         <v>57</v>
       </c>
@@ -4645,7 +4663,7 @@
       <c r="J58" s="10"/>
       <c r="K58" s="10"/>
     </row>
-    <row r="59" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="10">
         <v>58</v>
       </c>
@@ -4674,7 +4692,7 @@
       <c r="J59" s="10"/>
       <c r="K59" s="10"/>
     </row>
-    <row r="60" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="10">
         <v>59</v>
       </c>
@@ -4703,7 +4721,7 @@
       <c r="J60" s="10"/>
       <c r="K60" s="10"/>
     </row>
-    <row r="61" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" s="10">
         <v>60</v>
       </c>
@@ -4732,7 +4750,7 @@
       <c r="J61" s="10"/>
       <c r="K61" s="10"/>
     </row>
-    <row r="62" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62" s="10">
         <v>61</v>
       </c>
@@ -4761,7 +4779,7 @@
       <c r="J62" s="10"/>
       <c r="K62" s="10"/>
     </row>
-    <row r="63" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63" s="10">
         <v>62</v>
       </c>
@@ -4790,7 +4808,7 @@
       <c r="J63" s="10"/>
       <c r="K63" s="10"/>
     </row>
-    <row r="64" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="10">
         <v>63</v>
       </c>
@@ -4819,7 +4837,7 @@
       <c r="J64" s="10"/>
       <c r="K64" s="10"/>
     </row>
-    <row r="65" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="10">
         <v>64</v>
       </c>
@@ -4848,7 +4866,7 @@
       <c r="J65" s="10"/>
       <c r="K65" s="10"/>
     </row>
-    <row r="66" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="10">
         <v>65</v>
       </c>
@@ -4877,7 +4895,7 @@
       <c r="J66" s="10"/>
       <c r="K66" s="10"/>
     </row>
-    <row r="67" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="10">
         <v>66</v>
       </c>
@@ -4906,7 +4924,7 @@
       <c r="J67" s="10"/>
       <c r="K67" s="10"/>
     </row>
-    <row r="68" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="10">
         <v>67</v>
       </c>
@@ -4935,7 +4953,7 @@
       <c r="J68" s="10"/>
       <c r="K68" s="10"/>
     </row>
-    <row r="69" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="10">
         <v>68</v>
       </c>
@@ -4964,7 +4982,7 @@
       <c r="J69" s="10"/>
       <c r="K69" s="10"/>
     </row>
-    <row r="70" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="10">
         <v>69</v>
       </c>
@@ -4993,7 +5011,7 @@
       <c r="J70" s="10"/>
       <c r="K70" s="10"/>
     </row>
-    <row r="71" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="10">
         <v>70</v>
       </c>
@@ -5022,7 +5040,7 @@
       <c r="J71" s="10"/>
       <c r="K71" s="10"/>
     </row>
-    <row r="72" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="10">
         <v>71</v>
       </c>
@@ -5051,7 +5069,7 @@
       <c r="J72" s="10"/>
       <c r="K72" s="10"/>
     </row>
-    <row r="73" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="10">
         <v>72</v>
       </c>
@@ -5080,7 +5098,7 @@
       <c r="J73" s="10"/>
       <c r="K73" s="10"/>
     </row>
-    <row r="74" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="10">
         <v>73</v>
       </c>
@@ -5109,7 +5127,7 @@
       <c r="J74" s="10"/>
       <c r="K74" s="10"/>
     </row>
-    <row r="75" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="10">
         <v>74</v>
       </c>
@@ -5138,7 +5156,7 @@
       <c r="J75" s="10"/>
       <c r="K75" s="10"/>
     </row>
-    <row r="76" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="10">
         <v>75</v>
       </c>
@@ -5167,7 +5185,7 @@
       <c r="J76" s="10"/>
       <c r="K76" s="10"/>
     </row>
-    <row r="77" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="10">
         <v>76</v>
       </c>
@@ -5196,7 +5214,7 @@
       <c r="J77" s="10"/>
       <c r="K77" s="10"/>
     </row>
-    <row r="78" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="10">
         <v>77</v>
       </c>
@@ -5225,7 +5243,7 @@
       <c r="J78" s="10"/>
       <c r="K78" s="10"/>
     </row>
-    <row r="79" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="10">
         <v>78</v>
       </c>
@@ -5254,7 +5272,7 @@
       <c r="J79" s="10"/>
       <c r="K79" s="10"/>
     </row>
-    <row r="80" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="10">
         <v>79</v>
       </c>
@@ -5283,7 +5301,7 @@
       <c r="J80" s="10"/>
       <c r="K80" s="10"/>
     </row>
-    <row r="81" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="10">
         <v>80</v>
       </c>
@@ -5312,7 +5330,7 @@
       <c r="J81" s="10"/>
       <c r="K81" s="10"/>
     </row>
-    <row r="82" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="10">
         <v>81</v>
       </c>
@@ -5341,7 +5359,7 @@
       <c r="J82" s="10"/>
       <c r="K82" s="10"/>
     </row>
-    <row r="83" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="10">
         <v>82</v>
       </c>
@@ -5370,7 +5388,7 @@
       <c r="J83" s="10"/>
       <c r="K83" s="10"/>
     </row>
-    <row r="84" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="10">
         <v>83</v>
       </c>
@@ -5399,7 +5417,7 @@
       <c r="J84" s="10"/>
       <c r="K84" s="10"/>
     </row>
-    <row r="85" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="10">
         <v>84</v>
       </c>
@@ -5428,7 +5446,7 @@
       <c r="J85" s="10"/>
       <c r="K85" s="10"/>
     </row>
-    <row r="86" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="10">
         <v>85</v>
       </c>
@@ -5457,7 +5475,7 @@
       <c r="J86" s="10"/>
       <c r="K86" s="10"/>
     </row>
-    <row r="87" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="10">
         <v>86</v>
       </c>
@@ -5486,7 +5504,7 @@
       <c r="J87" s="10"/>
       <c r="K87" s="10"/>
     </row>
-    <row r="88" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="10">
         <v>87</v>
       </c>
@@ -5515,7 +5533,7 @@
       <c r="J88" s="10"/>
       <c r="K88" s="10"/>
     </row>
-    <row r="89" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="10">
         <v>88</v>
       </c>
@@ -5544,7 +5562,7 @@
       <c r="J89" s="10"/>
       <c r="K89" s="10"/>
     </row>
-    <row r="90" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A90" s="10">
         <v>89</v>
       </c>
@@ -5573,7 +5591,7 @@
       <c r="J90" s="10"/>
       <c r="K90" s="10"/>
     </row>
-    <row r="91" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" s="10">
         <v>90</v>
       </c>
@@ -5602,7 +5620,7 @@
       <c r="J91" s="10"/>
       <c r="K91" s="10"/>
     </row>
-    <row r="92" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="10">
         <v>91</v>
       </c>
@@ -5631,7 +5649,7 @@
       <c r="J92" s="10"/>
       <c r="K92" s="10"/>
     </row>
-    <row r="93" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="10">
         <v>92</v>
       </c>
@@ -5660,7 +5678,7 @@
       <c r="J93" s="10"/>
       <c r="K93" s="10"/>
     </row>
-    <row r="94" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="10">
         <v>93</v>
       </c>
@@ -5689,7 +5707,7 @@
       <c r="J94" s="10"/>
       <c r="K94" s="10"/>
     </row>
-    <row r="95" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="10">
         <v>94</v>
       </c>
@@ -5718,7 +5736,7 @@
       <c r="J95" s="10"/>
       <c r="K95" s="10"/>
     </row>
-    <row r="96" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="10">
         <v>95</v>
       </c>
@@ -5747,7 +5765,7 @@
       <c r="J96" s="10"/>
       <c r="K96" s="10"/>
     </row>
-    <row r="97" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97" s="10">
         <v>96</v>
       </c>
@@ -5776,7 +5794,7 @@
       <c r="J97" s="10"/>
       <c r="K97" s="10"/>
     </row>
-    <row r="98" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A98" s="10">
         <v>97</v>
       </c>
@@ -5805,7 +5823,7 @@
       <c r="J98" s="10"/>
       <c r="K98" s="10"/>
     </row>
-    <row r="99" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A99" s="10">
         <v>98</v>
       </c>
@@ -5834,7 +5852,7 @@
       <c r="J99" s="10"/>
       <c r="K99" s="10"/>
     </row>
-    <row r="100" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100" s="10">
         <v>99</v>
       </c>
@@ -5863,7 +5881,7 @@
       <c r="J100" s="10"/>
       <c r="K100" s="10"/>
     </row>
-    <row r="101" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101" s="10">
         <v>100</v>
       </c>
@@ -5892,7 +5910,7 @@
       <c r="J101" s="10"/>
       <c r="K101" s="10"/>
     </row>
-    <row r="102" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102" s="10">
         <v>101</v>
       </c>
@@ -5921,7 +5939,7 @@
       <c r="J102" s="10"/>
       <c r="K102" s="10"/>
     </row>
-    <row r="103" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103" s="10">
         <v>102</v>
       </c>
@@ -5950,7 +5968,7 @@
       <c r="J103" s="10"/>
       <c r="K103" s="10"/>
     </row>
-    <row r="104" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A104" s="10">
         <v>103</v>
       </c>
@@ -5979,7 +5997,7 @@
       <c r="J104" s="10"/>
       <c r="K104" s="10"/>
     </row>
-    <row r="105" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A105" s="10">
         <v>104</v>
       </c>
@@ -6008,7 +6026,7 @@
       <c r="J105" s="10"/>
       <c r="K105" s="10"/>
     </row>
-    <row r="106" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A106" s="10">
         <v>105</v>
       </c>
@@ -6037,7 +6055,7 @@
       <c r="J106" s="10"/>
       <c r="K106" s="10"/>
     </row>
-    <row r="107" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A107" s="10">
         <v>106</v>
       </c>
@@ -6066,7 +6084,7 @@
       <c r="J107" s="10"/>
       <c r="K107" s="10"/>
     </row>
-    <row r="108" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A108" s="10">
         <v>107</v>
       </c>
@@ -6095,7 +6113,7 @@
       <c r="J108" s="10"/>
       <c r="K108" s="10"/>
     </row>
-    <row r="109" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A109" s="10">
         <v>108</v>
       </c>
@@ -6124,7 +6142,7 @@
       <c r="J109" s="10"/>
       <c r="K109" s="10"/>
     </row>
-    <row r="110" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A110" s="10">
         <v>109</v>
       </c>
@@ -6153,7 +6171,7 @@
       <c r="J110" s="10"/>
       <c r="K110" s="10"/>
     </row>
-    <row r="111" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A111" s="10">
         <v>110</v>
       </c>
@@ -6183,32 +6201,32 @@
       <c r="K111" s="10"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K111"/>
+  <autoFilter ref="A1:K111" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <conditionalFormatting sqref="G2:G111">
+    <cfRule type="cellIs" dxfId="4" priority="6" operator="equal">
+      <formula>"High"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="H2:H111">
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="4" operator="equal">
       <formula>"Blocked"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="5" operator="equal">
       <formula>"Not Tested"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G111">
-    <cfRule type="cellIs" dxfId="0" priority="6" operator="equal">
-      <formula>"High"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" errorTitle="Invalid entry" error="Please choose a value from the list." sqref="H2:H111">
+    <dataValidation type="list" allowBlank="1" errorTitle="Invalid entry" error="Please choose a value from the list." sqref="H2:H111" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"Not Tested,Pass,Fail,Blocked,N/A"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="G2:G111">
+    <dataValidation type="list" allowBlank="1" sqref="G2:G111" xr:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>"High,Medium,Low"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
child daily log modified
</commit_message>
<xml_diff>
--- a/dc-uat-checklist.xlsx
+++ b/dc-uat-checklist.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\daycare-system\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49964668-5574-4B06-9A52-3BCB33A87CD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A168CA48-1F2A-4A2E-BCC7-75C5D25815AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="505">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="504">
   <si>
     <t>Emagine U At Play — UAT Checklist</t>
   </si>
@@ -1591,9 +1591,6 @@
   </si>
   <si>
     <t>None are present</t>
-  </si>
-  <si>
-    <t>Phone/mobile no placeholder issue</t>
   </si>
 </sst>
 </file>
@@ -2284,11 +2281,11 @@
       </c>
       <c r="D8" s="6">
         <f>COUNTIFS('UAT Checklist'!$B$2:$B$111,$B8,'UAT Checklist'!$H$2:$H$111,"Not Tested")</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E8" s="6">
         <f>COUNTIFS('UAT Checklist'!$B$2:$B$111,$B8,'UAT Checklist'!$H$2:$H$111,"Pass")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F8" s="6">
         <f>COUNTIFS('UAT Checklist'!$B$2:$B$111,$B8,'UAT Checklist'!$H$2:$H$111,"Fail")</f>
@@ -2304,7 +2301,7 @@
       </c>
       <c r="I8" s="7">
         <f t="shared" si="0"/>
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.35">
@@ -2911,11 +2908,11 @@
       </c>
       <c r="D27" s="8">
         <f t="shared" si="1"/>
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E27" s="8">
         <f t="shared" si="1"/>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F27" s="8">
         <f t="shared" si="1"/>
@@ -2931,7 +2928,7 @@
       </c>
       <c r="I27" s="9">
         <f t="shared" si="0"/>
-        <v>0.11818181818181818</v>
+        <v>0.13636363636363635</v>
       </c>
     </row>
   </sheetData>
@@ -3033,9 +3030,7 @@
       <c r="H2" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="11" t="s">
-        <v>504</v>
-      </c>
+      <c r="I2" s="11"/>
       <c r="J2" s="10"/>
       <c r="K2" s="10"/>
     </row>
@@ -3468,7 +3463,7 @@
         <v>67</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I17" s="11"/>
       <c r="J17" s="10"/>
@@ -3497,7 +3492,7 @@
         <v>67</v>
       </c>
       <c r="H18" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I18" s="11"/>
       <c r="J18" s="10"/>

</xml_diff>